<commit_message>
Added scholar orient unlocks
</commit_message>
<xml_diff>
--- a/data/config/export/main/asset/excel/Unlocks.xlsx
+++ b/data/config/export/main/asset/excel/Unlocks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Max\Documents\Anno 1800\mods\[Addon] Return to the Orient\data\config\export\main\asset\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0174CC9F-B534-4358-A022-BB9B76E42CC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDF30F61-A74E-474A-B854-6659BE87B181}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="5235" windowWidth="29040" windowHeight="16440" xr2:uid="{44479434-C7CF-4AB1-AF8F-C5342A9CF046}"/>
   </bookViews>
@@ -18,7 +18,7 @@
     <sheet name="Vanilla" sheetId="2" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Orient!$A$1:$D$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Orient!$A$1:$D$54</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Vanilla!$A$1:$G$10</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="125">
   <si>
     <t>Name</t>
   </si>
@@ -424,7 +424,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -468,8 +468,53 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="4"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -486,8 +531,20 @@
         <fgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -513,6 +570,77 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -520,7 +648,7 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -532,7 +660,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="2" borderId="0" xfId="2" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -571,6 +698,59 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="3" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Bad" xfId="3" builtinId="27"/>
@@ -888,7 +1068,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3D4DA87-30D8-4E7C-A972-205573E34910}">
-  <dimension ref="A1:D59"/>
+  <dimension ref="A1:H58"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.5703125" style="1" bestFit="1" customWidth="1"/>
@@ -1111,7 +1291,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>19</v>
       </c>
@@ -1125,36 +1305,42 @@
         <v>300</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="7" t="s">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D18" s="11">
+      <c r="D18" s="4">
         <v>300</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="34" t="s">
         <v>47</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="35" t="s">
         <v>48</v>
       </c>
-      <c r="C19" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D19" s="4">
+      <c r="C19" s="35" t="s">
+        <v>13</v>
+      </c>
+      <c r="D19" s="54">
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
+      <c r="E19" s="36">
+        <v>1</v>
+      </c>
+      <c r="F19" s="79">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="37" t="s">
         <v>44</v>
       </c>
       <c r="C20" s="1" t="s">
@@ -1163,51 +1349,73 @@
       <c r="D20" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
+      <c r="E20" s="38">
+        <v>1</v>
+      </c>
+      <c r="F20" s="79"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="48" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="C21" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D21" s="4">
+      <c r="C21" s="29" t="s">
+        <v>13</v>
+      </c>
+      <c r="D21" s="30">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="D22" s="6">
+      <c r="E21" s="38">
         <v>1</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
+      <c r="F21" s="79"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="52" t="s">
+        <v>22</v>
+      </c>
+      <c r="B22" s="53" t="s">
+        <v>10</v>
+      </c>
+      <c r="C22" s="53" t="s">
+        <v>13</v>
+      </c>
+      <c r="D22" s="53">
+        <v>300</v>
+      </c>
+      <c r="E22" s="42">
+        <v>1</v>
+      </c>
+      <c r="F22" s="79"/>
+      <c r="G22" s="1"/>
+      <c r="H22" s="1"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="34" t="s">
         <v>40</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="C23" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D23" s="1">
+      <c r="C23" s="35" t="s">
+        <v>13</v>
+      </c>
+      <c r="D23" s="35">
         <v>300</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
+      <c r="E23" s="36">
+        <v>300</v>
+      </c>
+      <c r="F23" s="79">
+        <v>1</v>
+      </c>
+      <c r="G23" s="1"/>
+      <c r="H23" s="1"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="37" t="s">
         <v>41</v>
       </c>
       <c r="B24" s="1" t="s">
@@ -1219,9 +1427,15 @@
       <c r="D24" s="1">
         <v>300</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
+      <c r="E24" s="38">
+        <v>300</v>
+      </c>
+      <c r="F24" s="79"/>
+      <c r="G24" s="1"/>
+      <c r="H24" s="1"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="37" t="s">
         <v>52</v>
       </c>
       <c r="C25" s="1" t="s">
@@ -1230,24 +1444,35 @@
       <c r="D25" s="1">
         <v>300</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D26" s="1">
+      <c r="E25" s="38">
         <v>300</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="5" t="s">
+      <c r="F25" s="79"/>
+      <c r="G25" s="1"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="39" t="s">
         <v>55</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D26" s="5">
+        <v>300</v>
+      </c>
+      <c r="E26" s="38">
+        <v>300</v>
+      </c>
+      <c r="F26" s="79"/>
+      <c r="G26" s="1"/>
+      <c r="H26" s="1"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="39" t="s">
+        <v>56</v>
       </c>
       <c r="B27" s="5" t="s">
         <v>51</v>
@@ -1258,426 +1483,626 @@
       <c r="D27" s="5">
         <v>300</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B28" s="6" t="s">
+      <c r="E27" s="38">
+        <v>300</v>
+      </c>
+      <c r="F27" s="79"/>
+      <c r="G27" s="1"/>
+      <c r="H27" s="1"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="40" t="s">
+        <v>26</v>
+      </c>
+      <c r="B28" s="33" t="s">
+        <v>11</v>
+      </c>
+      <c r="C28" s="33" t="s">
+        <v>13</v>
+      </c>
+      <c r="D28" s="33">
+        <v>600</v>
+      </c>
+      <c r="E28" s="38">
+        <v>300</v>
+      </c>
+      <c r="F28" s="79"/>
+      <c r="G28" s="1"/>
+      <c r="H28" s="1"/>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="41" t="s">
+        <v>53</v>
+      </c>
+      <c r="B29" s="2"/>
+      <c r="C29" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D29" s="2">
+        <v>600</v>
+      </c>
+      <c r="E29" s="42">
+        <v>300</v>
+      </c>
+      <c r="F29" s="79"/>
+      <c r="G29" s="1"/>
+      <c r="H29" s="1"/>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="60" t="s">
+        <v>57</v>
+      </c>
+      <c r="B30" s="61" t="s">
+        <v>48</v>
+      </c>
+      <c r="C30" s="61" t="s">
+        <v>13</v>
+      </c>
+      <c r="D30" s="61">
+        <v>600</v>
+      </c>
+      <c r="E30" s="62">
+        <v>600</v>
+      </c>
+      <c r="F30" s="79">
+        <v>2</v>
+      </c>
+      <c r="G30" s="1"/>
+      <c r="H30" s="1"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" s="46" t="s">
+        <v>2</v>
+      </c>
+      <c r="B31" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="C31" s="31" t="s">
+        <v>13</v>
+      </c>
+      <c r="D31" s="32">
+        <v>600</v>
+      </c>
+      <c r="E31" s="63">
+        <v>600</v>
+      </c>
+      <c r="F31" s="79"/>
+      <c r="G31" s="1"/>
+      <c r="H31" s="1"/>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" s="46" t="s">
+        <v>3</v>
+      </c>
+      <c r="B32" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="C32" s="31" t="s">
+        <v>13</v>
+      </c>
+      <c r="D32" s="32">
+        <v>600</v>
+      </c>
+      <c r="E32" s="63">
+        <v>600</v>
+      </c>
+      <c r="F32" s="79"/>
+      <c r="G32" s="1"/>
+      <c r="H32" s="1"/>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" s="64" t="s">
+        <v>24</v>
+      </c>
+      <c r="B33" s="65" t="s">
+        <v>10</v>
+      </c>
+      <c r="C33" s="65" t="s">
+        <v>13</v>
+      </c>
+      <c r="D33" s="65">
+        <v>1000</v>
+      </c>
+      <c r="E33" s="63">
+        <v>600</v>
+      </c>
+      <c r="F33" s="79"/>
+      <c r="G33" s="1"/>
+      <c r="H33" s="1"/>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" s="48" t="s">
+        <v>25</v>
+      </c>
+      <c r="B34" s="29" t="s">
+        <v>10</v>
+      </c>
+      <c r="C34" s="29" t="s">
+        <v>13</v>
+      </c>
+      <c r="D34" s="29">
+        <v>1000</v>
+      </c>
+      <c r="E34" s="63">
+        <v>600</v>
+      </c>
+      <c r="F34" s="79"/>
+      <c r="G34" s="1"/>
+      <c r="H34" s="1"/>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" s="66" t="s">
+        <v>58</v>
+      </c>
+      <c r="B35" s="67" t="s">
         <v>51</v>
       </c>
-      <c r="C28" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="D28" s="6">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="29" t="s">
-        <v>26</v>
-      </c>
-      <c r="B29" s="29" t="s">
+      <c r="C35" s="67" t="s">
+        <v>13</v>
+      </c>
+      <c r="D35" s="67">
+        <v>1000</v>
+      </c>
+      <c r="E35" s="68">
+        <v>600</v>
+      </c>
+      <c r="F35" s="79"/>
+      <c r="G35" s="1"/>
+      <c r="H35" s="1"/>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" s="69" t="s">
+        <v>4</v>
+      </c>
+      <c r="B36" s="70" t="s">
         <v>11</v>
       </c>
-      <c r="C29" s="29" t="s">
-        <v>13</v>
-      </c>
-      <c r="D29" s="29">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D30" s="1">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="B31" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="C31" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D31" s="5">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B32" s="1" t="s">
+      <c r="C36" s="70" t="s">
+        <v>13</v>
+      </c>
+      <c r="D36" s="70">
+        <v>1400</v>
+      </c>
+      <c r="E36" s="55">
+        <v>1000</v>
+      </c>
+      <c r="F36" s="79">
+        <v>3</v>
+      </c>
+      <c r="G36" s="1"/>
+      <c r="H36" s="1"/>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" s="56" t="s">
+        <v>5</v>
+      </c>
+      <c r="B37" s="57" t="s">
         <v>11</v>
       </c>
-      <c r="C32" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D32" s="4">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B33" s="2" t="s">
+      <c r="C37" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="D37" s="57">
+        <v>1400</v>
+      </c>
+      <c r="E37" s="58">
+        <v>1000</v>
+      </c>
+      <c r="F37" s="79"/>
+      <c r="G37" s="1"/>
+      <c r="H37" s="1"/>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" s="71" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38" s="72" t="s">
+        <v>51</v>
+      </c>
+      <c r="C38" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="D38" s="72">
+        <v>1400</v>
+      </c>
+      <c r="E38" s="58">
+        <v>1000</v>
+      </c>
+      <c r="F38" s="79"/>
+      <c r="G38" s="1"/>
+      <c r="H38" s="1"/>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A39" s="71" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39" s="72" t="s">
+        <v>51</v>
+      </c>
+      <c r="C39" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="D39" s="72">
+        <v>1400</v>
+      </c>
+      <c r="E39" s="58">
+        <v>1000</v>
+      </c>
+      <c r="F39" s="79"/>
+      <c r="G39" s="1"/>
+      <c r="H39" s="1"/>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A40" s="73" t="s">
+        <v>27</v>
+      </c>
+      <c r="B40" s="74" t="s">
+        <v>10</v>
+      </c>
+      <c r="C40" s="74" t="s">
+        <v>13</v>
+      </c>
+      <c r="D40" s="74">
+        <v>1900</v>
+      </c>
+      <c r="E40" s="59">
+        <v>1000</v>
+      </c>
+      <c r="F40" s="79"/>
+      <c r="G40" s="1"/>
+      <c r="H40" s="1"/>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A41" s="50" t="s">
+        <v>6</v>
+      </c>
+      <c r="B41" s="51" t="s">
         <v>11</v>
       </c>
-      <c r="C33" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D33" s="9">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B34" s="1" t="s">
+      <c r="C41" s="51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D41" s="51">
+        <v>1900</v>
+      </c>
+      <c r="E41" s="45">
+        <v>1400</v>
+      </c>
+      <c r="F41" s="79">
+        <v>4</v>
+      </c>
+      <c r="G41" s="1"/>
+      <c r="H41" s="1"/>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A42" s="46" t="s">
+        <v>7</v>
+      </c>
+      <c r="B42" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="C42" s="31" t="s">
+        <v>13</v>
+      </c>
+      <c r="D42" s="31">
+        <v>1900</v>
+      </c>
+      <c r="E42" s="47">
+        <v>1400</v>
+      </c>
+      <c r="F42" s="79"/>
+      <c r="G42" s="1"/>
+      <c r="H42" s="1"/>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43" s="39" t="s">
+        <v>61</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D43" s="5">
+        <v>1900</v>
+      </c>
+      <c r="E43" s="47">
+        <v>1400</v>
+      </c>
+      <c r="F43" s="79"/>
+      <c r="G43" s="1"/>
+      <c r="H43" s="1"/>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A44" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="B44" s="53" t="s">
         <v>10</v>
       </c>
-      <c r="C34" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D34" s="1">
+      <c r="C44" s="53" t="s">
+        <v>13</v>
+      </c>
+      <c r="D44" s="53">
+        <v>2400</v>
+      </c>
+      <c r="E44" s="49">
+        <v>1400</v>
+      </c>
+      <c r="F44" s="79"/>
+      <c r="G44" s="1"/>
+      <c r="H44" s="1"/>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45" s="43" t="s">
+        <v>62</v>
+      </c>
+      <c r="B45" s="44" t="s">
+        <v>51</v>
+      </c>
+      <c r="C45" s="44" t="s">
+        <v>13</v>
+      </c>
+      <c r="D45" s="44">
+        <v>2400</v>
+      </c>
+      <c r="E45" s="36">
+        <v>1900</v>
+      </c>
+      <c r="F45" s="79">
+        <v>5</v>
+      </c>
+      <c r="G45" s="1"/>
+      <c r="H45" s="1"/>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46" s="46" t="s">
+        <v>8</v>
+      </c>
+      <c r="B46" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="C46" s="31" t="s">
+        <v>13</v>
+      </c>
+      <c r="D46" s="31">
+        <v>3000</v>
+      </c>
+      <c r="E46" s="38">
+        <v>1900</v>
+      </c>
+      <c r="F46" s="79"/>
+      <c r="G46" s="1"/>
+      <c r="H46" s="1"/>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A47" s="46" t="s">
+        <v>9</v>
+      </c>
+      <c r="B47" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="C47" s="31" t="s">
+        <v>13</v>
+      </c>
+      <c r="D47" s="31">
+        <v>3000</v>
+      </c>
+      <c r="E47" s="38">
+        <v>1900</v>
+      </c>
+      <c r="F47" s="79"/>
+      <c r="G47" s="1"/>
+      <c r="H47" s="1"/>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A48" s="41" t="s">
+        <v>77</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D48" s="2">
+        <v>3000</v>
+      </c>
+      <c r="E48" s="42">
+        <v>1900</v>
+      </c>
+      <c r="F48" s="79"/>
+      <c r="G48" s="1"/>
+      <c r="H48" s="1"/>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A49" s="75" t="s">
+        <v>30</v>
+      </c>
+      <c r="B49" s="76" t="s">
+        <v>10</v>
+      </c>
+      <c r="C49" s="76" t="s">
+        <v>13</v>
+      </c>
+      <c r="D49" s="76">
+        <v>3600</v>
+      </c>
+      <c r="E49" s="45">
+        <v>2400</v>
+      </c>
+      <c r="F49" s="79">
+        <v>6</v>
+      </c>
+      <c r="G49" s="1"/>
+      <c r="H49" s="1"/>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A50" s="41" t="s">
+        <v>78</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D50" s="2">
+        <v>3600</v>
+      </c>
+      <c r="E50" s="49">
+        <v>2400</v>
+      </c>
+      <c r="F50" s="79"/>
+      <c r="G50" s="1"/>
+      <c r="H50" s="1"/>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A51" s="77" t="s">
+        <v>31</v>
+      </c>
+      <c r="B51" s="78" t="s">
+        <v>11</v>
+      </c>
+      <c r="C51" s="78" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51" s="78">
+        <v>4300</v>
+      </c>
+      <c r="E51" s="45">
+        <v>3000</v>
+      </c>
+      <c r="F51" s="79">
+        <v>7</v>
+      </c>
+      <c r="G51" s="1"/>
+      <c r="H51" s="1"/>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A52" s="41" t="s">
+        <v>79</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D52" s="2">
+        <v>4300</v>
+      </c>
+      <c r="E52" s="49">
+        <v>3000</v>
+      </c>
+      <c r="F52" s="79"/>
+      <c r="G52" s="1"/>
+      <c r="H52" s="1"/>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A53" s="75" t="s">
+        <v>32</v>
+      </c>
+      <c r="B53" s="76" t="s">
+        <v>10</v>
+      </c>
+      <c r="C53" s="76" t="s">
+        <v>13</v>
+      </c>
+      <c r="D53" s="76">
+        <v>5000</v>
+      </c>
+      <c r="E53" s="45">
+        <v>3600</v>
+      </c>
+      <c r="F53" s="79">
+        <v>8</v>
+      </c>
+      <c r="G53" s="1"/>
+      <c r="H53" s="1"/>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A54" s="41" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D54" s="2">
+        <v>5000</v>
+      </c>
+      <c r="E54" s="49">
+        <v>3600</v>
+      </c>
+      <c r="F54" s="79"/>
+      <c r="G54" s="1"/>
+      <c r="H54" s="1"/>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A55" s="28" t="s">
+        <v>23</v>
+      </c>
+      <c r="B55" s="28" t="s">
+        <v>10</v>
+      </c>
+      <c r="C55" s="28" t="s">
+        <v>124</v>
+      </c>
+      <c r="D55" s="28">
         <v>1000</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B35" s="1" t="s">
+      <c r="E55" s="1"/>
+      <c r="F55" s="1"/>
+      <c r="G55" s="1"/>
+      <c r="H55" s="1"/>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A56" s="28" t="s">
+        <v>29</v>
+      </c>
+      <c r="B56" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="C35" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D35" s="1">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="B36" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="C36" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="D36" s="6">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D37" s="1">
-        <v>1400</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D38" s="1">
-        <v>1400</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="B40" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C40" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D40" s="5">
-        <v>1400</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="B41" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="C41" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="D41" s="6">
-        <v>1400</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B42" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C42" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D42" s="1">
-        <v>1900</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B43" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D43" s="1">
-        <v>1900</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D44" s="1">
-        <v>1900</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="B45" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="C45" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="D45" s="6">
-        <v>1900</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B46" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C46" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D46" s="1">
-        <v>2400</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="B48" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="C48" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="D48" s="6">
-        <v>2400</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B49" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C49" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D49" s="1">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B50" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C50" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D50" s="1">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B51" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C51" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D51" s="2">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B52" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C52" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D52" s="1">
-        <v>3600</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="B53" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C53" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D53" s="2">
-        <v>3600</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B54" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C54" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D54" s="1">
-        <v>4300</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="B55" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D55" s="2">
-        <v>4300</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B56" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C56" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D56" s="1">
-        <v>5000</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="B57" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C57" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D57" s="2">
-        <v>5000</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="29" t="s">
-        <v>23</v>
-      </c>
-      <c r="B58" s="29" t="s">
-        <v>10</v>
-      </c>
-      <c r="C58" s="29" t="s">
+      <c r="C56" s="28" t="s">
         <v>124</v>
       </c>
-      <c r="D58" s="29">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="29" t="s">
-        <v>29</v>
-      </c>
-      <c r="B59" s="29" t="s">
-        <v>10</v>
-      </c>
-      <c r="C59" s="29" t="s">
-        <v>124</v>
-      </c>
-      <c r="D59" s="29">
+      <c r="D56" s="28">
         <v>7000</v>
       </c>
+      <c r="E56" s="1"/>
+      <c r="F56" s="1"/>
+      <c r="G56" s="1"/>
+      <c r="H56" s="1"/>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E57" s="1"/>
+      <c r="F57" s="1"/>
+      <c r="G57" s="1"/>
+      <c r="H57" s="1"/>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E58" s="1"/>
+      <c r="F58" s="1"/>
+      <c r="G58" s="1"/>
+      <c r="H58" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D57" xr:uid="{E3D4DA87-30D8-4E7C-A972-205573E34910}"/>
+  <autoFilter ref="A1:D56" xr:uid="{E3D4DA87-30D8-4E7C-A972-205573E34910}"/>
+  <mergeCells count="9">
+    <mergeCell ref="F49:F50"/>
+    <mergeCell ref="F51:F52"/>
+    <mergeCell ref="F53:F54"/>
+    <mergeCell ref="F19:F22"/>
+    <mergeCell ref="F23:F29"/>
+    <mergeCell ref="F30:F35"/>
+    <mergeCell ref="F36:F40"/>
+    <mergeCell ref="F41:F44"/>
+    <mergeCell ref="F45:F48"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -1691,8 +2116,8 @@
     <col min="1" max="1" width="10.28515625" customWidth="1"/>
     <col min="2" max="2" width="38.28515625" customWidth="1"/>
     <col min="3" max="3" width="12.42578125" customWidth="1"/>
-    <col min="4" max="4" width="12.42578125" style="28" customWidth="1"/>
-    <col min="5" max="5" width="15.5703125" style="15" customWidth="1"/>
+    <col min="4" max="4" width="12.42578125" style="27" customWidth="1"/>
+    <col min="5" max="5" width="15.5703125" style="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:5" s="10" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1702,110 +2127,110 @@
       <c r="C2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="19" t="s">
+      <c r="D2" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="14" t="s">
+      <c r="E2" s="13" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="3" spans="1:5" s="13" customFormat="1" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="12" t="s">
+    <row r="3" spans="1:5" s="12" customFormat="1" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="11" t="s">
         <v>120</v>
       </c>
-      <c r="D3" s="20">
+      <c r="D3" s="19">
         <v>0</v>
       </c>
-      <c r="E3" s="15">
+      <c r="E3" s="14">
         <v>1404000000</v>
       </c>
     </row>
-    <row r="4" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="12" t="s">
+    <row r="4" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="D4" s="20">
+      <c r="D4" s="19">
         <v>0</v>
       </c>
-      <c r="E4" s="15">
+      <c r="E4" s="14">
         <v>1404000014</v>
       </c>
     </row>
-    <row r="5" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="12" t="s">
+    <row r="5" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="D5" s="20">
+      <c r="D5" s="19">
         <v>0</v>
       </c>
-      <c r="E5" s="15">
+      <c r="E5" s="14">
         <v>1404000614</v>
       </c>
     </row>
-    <row r="6" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="12" t="s">
+    <row r="6" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="D6" s="20">
+      <c r="D6" s="19">
         <v>0</v>
       </c>
-      <c r="E6" s="15">
+      <c r="E6" s="14">
         <v>1404000616</v>
       </c>
     </row>
-    <row r="7" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="12" t="s">
+    <row r="7" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="D7" s="20">
+      <c r="D7" s="19">
         <v>0</v>
       </c>
-      <c r="E7" s="15">
+      <c r="E7" s="14">
         <v>1404000617</v>
       </c>
     </row>
-    <row r="8" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="12" t="s">
+    <row r="8" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="D8" s="20">
+      <c r="D8" s="19">
         <v>0</v>
       </c>
-      <c r="E8" s="15">
+      <c r="E8" s="14">
         <v>1404000618</v>
       </c>
     </row>
-    <row r="9" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="12" t="s">
+    <row r="9" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="D9" s="20">
+      <c r="D9" s="19">
         <v>0</v>
       </c>
-      <c r="E9" s="15">
+      <c r="E9" s="14">
         <v>1404000619</v>
       </c>
     </row>
-    <row r="10" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="12" t="s">
+    <row r="10" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="D10" s="20">
+      <c r="D10" s="19">
         <v>0</v>
       </c>
-      <c r="E10" s="15">
+      <c r="E10" s="14">
         <v>1404000620</v>
       </c>
     </row>
-    <row r="11" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>121</v>
       </c>
       <c r="C11"/>
-      <c r="D11" s="20">
+      <c r="D11" s="19">
         <v>0</v>
       </c>
-      <c r="E11" s="15">
+      <c r="E11" s="14">
         <v>1404000218</v>
       </c>
     </row>
@@ -1817,10 +2242,10 @@
       <c r="C12" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D12" s="21">
+      <c r="D12" s="20">
         <v>0</v>
       </c>
-      <c r="E12" s="15">
+      <c r="E12" s="14">
         <v>114523</v>
       </c>
     </row>
@@ -1832,10 +2257,10 @@
       <c r="C13" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D13" s="21">
+      <c r="D13" s="20">
         <v>0</v>
       </c>
-      <c r="E13" s="15">
+      <c r="E13" s="14">
         <v>1404000790</v>
       </c>
     </row>
@@ -1845,10 +2270,10 @@
         <v>123</v>
       </c>
       <c r="C14" s="1"/>
-      <c r="D14" s="21">
+      <c r="D14" s="20">
         <v>0</v>
       </c>
-      <c r="E14" s="15">
+      <c r="E14" s="14">
         <v>1404000016</v>
       </c>
     </row>
@@ -1856,10 +2281,10 @@
       <c r="B15" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D15" s="22">
+      <c r="D15" s="21">
         <v>0</v>
       </c>
-      <c r="E15" s="16">
+      <c r="E15" s="15">
         <v>1404000156</v>
       </c>
     </row>
@@ -1871,10 +2296,10 @@
       <c r="C16" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D16" s="23">
+      <c r="D16" s="22">
         <v>50</v>
       </c>
-      <c r="E16" s="15" t="s">
+      <c r="E16" s="14" t="s">
         <v>94</v>
       </c>
     </row>
@@ -1885,21 +2310,21 @@
       <c r="C17" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D17" s="22">
+      <c r="D17" s="21">
         <v>50</v>
       </c>
-      <c r="E17" s="16" t="s">
+      <c r="E17" s="15" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="18" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="12" t="s">
+      <c r="B18" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="D18" s="23">
+      <c r="D18" s="22">
         <v>100</v>
       </c>
-      <c r="E18" s="15">
+      <c r="E18" s="14">
         <v>1404000215</v>
       </c>
     </row>
@@ -1911,10 +2336,10 @@
       <c r="C19" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D19" s="23">
+      <c r="D19" s="22">
         <v>100</v>
       </c>
-      <c r="E19" s="15">
+      <c r="E19" s="14">
         <v>101339</v>
       </c>
     </row>
@@ -1926,10 +2351,10 @@
       <c r="C20" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D20" s="23">
+      <c r="D20" s="22">
         <v>100</v>
       </c>
-      <c r="E20" s="15">
+      <c r="E20" s="14">
         <v>1404000217</v>
       </c>
     </row>
@@ -1941,10 +2366,10 @@
       <c r="C21" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D21" s="23">
+      <c r="D21" s="22">
         <v>100</v>
       </c>
-      <c r="E21" s="15" t="s">
+      <c r="E21" s="14" t="s">
         <v>95</v>
       </c>
     </row>
@@ -1954,10 +2379,10 @@
         <v>46</v>
       </c>
       <c r="C22" s="1"/>
-      <c r="D22" s="23">
+      <c r="D22" s="22">
         <v>100</v>
       </c>
-      <c r="E22" s="15">
+      <c r="E22" s="14">
         <v>1404000376</v>
       </c>
     </row>
@@ -1969,10 +2394,10 @@
       <c r="C23" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D23" s="23">
+      <c r="D23" s="22">
         <v>100</v>
       </c>
-      <c r="E23" s="15" t="s">
+      <c r="E23" s="14" t="s">
         <v>117</v>
       </c>
     </row>
@@ -1983,10 +2408,10 @@
       <c r="C24" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="D24" s="24">
+      <c r="D24" s="23">
         <v>100</v>
       </c>
-      <c r="E24" s="16">
+      <c r="E24" s="15">
         <v>1404000379</v>
       </c>
     </row>
@@ -1996,10 +2421,10 @@
         <v>44</v>
       </c>
       <c r="C25" s="1"/>
-      <c r="D25" s="23">
+      <c r="D25" s="22">
         <v>200</v>
       </c>
-      <c r="E25" s="15" t="s">
+      <c r="E25" s="14" t="s">
         <v>96</v>
       </c>
     </row>
@@ -2009,10 +2434,10 @@
         <v>45</v>
       </c>
       <c r="C26" s="1"/>
-      <c r="D26" s="23">
+      <c r="D26" s="22">
         <v>200</v>
       </c>
-      <c r="E26" s="15">
+      <c r="E26" s="14">
         <v>1404000203</v>
       </c>
     </row>
@@ -2023,10 +2448,10 @@
       <c r="C27" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="D27" s="25">
+      <c r="D27" s="24">
         <v>200</v>
       </c>
-      <c r="E27" s="16">
+      <c r="E27" s="15">
         <v>133886</v>
       </c>
     </row>
@@ -2038,10 +2463,10 @@
       <c r="C28" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D28" s="23">
+      <c r="D28" s="22">
         <v>300</v>
       </c>
-      <c r="E28" s="17" t="s">
+      <c r="E28" s="16" t="s">
         <v>97</v>
       </c>
     </row>
@@ -2053,10 +2478,10 @@
       <c r="C29" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D29" s="23">
+      <c r="D29" s="22">
         <v>300</v>
       </c>
-      <c r="E29" s="17" t="s">
+      <c r="E29" s="16" t="s">
         <v>98</v>
       </c>
     </row>
@@ -2067,18 +2492,18 @@
       <c r="D30" s="7">
         <v>300</v>
       </c>
-      <c r="E30" s="18">
+      <c r="E30" s="17">
         <v>1404000017</v>
       </c>
     </row>
     <row r="31" spans="1:5" s="1" customFormat="1" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="12" t="s">
+      <c r="B31" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="D31" s="23">
+      <c r="D31" s="22">
         <v>1</v>
       </c>
-      <c r="E31" s="15">
+      <c r="E31" s="14">
         <v>1404000015</v>
       </c>
     </row>
@@ -2090,10 +2515,10 @@
       <c r="C32" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D32" s="23">
+      <c r="D32" s="22">
         <v>1</v>
       </c>
-      <c r="E32" s="15">
+      <c r="E32" s="14">
         <v>119029</v>
       </c>
     </row>
@@ -2105,23 +2530,23 @@
       <c r="C33" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D33" s="23">
+      <c r="D33" s="22">
         <v>1</v>
       </c>
-      <c r="E33" s="15" t="s">
+      <c r="E33" s="14" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
-      <c r="B34" s="12" t="s">
+      <c r="B34" s="11" t="s">
         <v>83</v>
       </c>
       <c r="C34" s="1"/>
-      <c r="D34" s="23">
+      <c r="D34" s="22">
         <v>1</v>
       </c>
-      <c r="E34" s="17">
+      <c r="E34" s="16">
         <v>1404000372</v>
       </c>
       <c r="F34">
@@ -2136,10 +2561,10 @@
       <c r="C35" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D35" s="23">
+      <c r="D35" s="22">
         <v>1</v>
       </c>
-      <c r="E35" s="17" t="s">
+      <c r="E35" s="16" t="s">
         <v>100</v>
       </c>
     </row>
@@ -2150,22 +2575,22 @@
       <c r="C36" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D36" s="22">
+      <c r="D36" s="21">
         <v>1</v>
       </c>
-      <c r="E36" s="16" t="s">
+      <c r="E36" s="15" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="37" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="12" t="s">
+      <c r="B37" s="11" t="s">
         <v>85</v>
       </c>
       <c r="C37" s="5"/>
-      <c r="D37" s="21">
+      <c r="D37" s="20">
         <v>300</v>
       </c>
-      <c r="E37" s="15">
+      <c r="E37" s="14">
         <v>1404000615</v>
       </c>
     </row>
@@ -2177,10 +2602,10 @@
       <c r="C38" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D38" s="21">
+      <c r="D38" s="20">
         <v>300</v>
       </c>
-      <c r="E38" s="15">
+      <c r="E38" s="14">
         <v>101573</v>
       </c>
     </row>
@@ -2192,10 +2617,10 @@
       <c r="C39" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D39" s="21">
+      <c r="D39" s="20">
         <v>300</v>
       </c>
-      <c r="E39" s="15">
+      <c r="E39" s="14">
         <v>101344</v>
       </c>
     </row>
@@ -2205,10 +2630,10 @@
         <v>52</v>
       </c>
       <c r="C40" s="1"/>
-      <c r="D40" s="21">
+      <c r="D40" s="20">
         <v>300</v>
       </c>
-      <c r="E40" s="15">
+      <c r="E40" s="14">
         <v>1404000202</v>
       </c>
       <c r="F40">
@@ -2223,10 +2648,10 @@
       <c r="C41" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D41" s="21">
+      <c r="D41" s="20">
         <v>300</v>
       </c>
-      <c r="E41" s="15" t="s">
+      <c r="E41" s="14" t="s">
         <v>102</v>
       </c>
     </row>
@@ -2238,10 +2663,10 @@
       <c r="C42" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="D42" s="26">
+      <c r="D42" s="25">
         <v>300</v>
       </c>
-      <c r="E42" s="15">
+      <c r="E42" s="14">
         <v>1404000584</v>
       </c>
     </row>
@@ -2252,10 +2677,10 @@
       <c r="C43" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="D43" s="25">
+      <c r="D43" s="24">
         <v>300</v>
       </c>
-      <c r="E43" s="16">
+      <c r="E43" s="15">
         <v>1404000585</v>
       </c>
     </row>
@@ -2267,10 +2692,10 @@
       <c r="C44" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D44" s="21">
+      <c r="D44" s="20">
         <v>600</v>
       </c>
-      <c r="E44" s="15" t="s">
+      <c r="E44" s="14" t="s">
         <v>103</v>
       </c>
     </row>
@@ -2280,10 +2705,10 @@
         <v>53</v>
       </c>
       <c r="C45" s="1"/>
-      <c r="D45" s="21">
+      <c r="D45" s="20">
         <v>600</v>
       </c>
-      <c r="E45" s="15">
+      <c r="E45" s="14">
         <v>1404000375</v>
       </c>
       <c r="F45">
@@ -2297,10 +2722,10 @@
       <c r="C46" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="D46" s="25">
+      <c r="D46" s="24">
         <v>600</v>
       </c>
-      <c r="E46" s="16">
+      <c r="E46" s="15">
         <v>1404000380</v>
       </c>
     </row>
@@ -2312,10 +2737,10 @@
       <c r="C47" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D47" s="21">
+      <c r="D47" s="20">
         <v>1000</v>
       </c>
-      <c r="E47" s="15" t="s">
+      <c r="E47" s="14" t="s">
         <v>104</v>
       </c>
     </row>
@@ -2327,10 +2752,10 @@
       <c r="C48" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D48" s="21">
+      <c r="D48" s="20">
         <v>1000</v>
       </c>
-      <c r="E48" s="15" t="s">
+      <c r="E48" s="14" t="s">
         <v>105</v>
       </c>
       <c r="F48">
@@ -2344,10 +2769,10 @@
       <c r="C49" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="D49" s="25">
+      <c r="D49" s="24">
         <v>1000</v>
       </c>
-      <c r="E49" s="16">
+      <c r="E49" s="15">
         <v>1404000381</v>
       </c>
     </row>
@@ -2359,10 +2784,10 @@
       <c r="C50" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D50" s="21">
+      <c r="D50" s="20">
         <v>1400</v>
       </c>
-      <c r="E50" s="15" t="s">
+      <c r="E50" s="14" t="s">
         <v>106</v>
       </c>
     </row>
@@ -2374,10 +2799,10 @@
       <c r="C51" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D51" s="21">
+      <c r="D51" s="20">
         <v>1400</v>
       </c>
-      <c r="E51" s="15" t="s">
+      <c r="E51" s="14" t="s">
         <v>107</v>
       </c>
       <c r="F51">
@@ -2392,10 +2817,10 @@
       <c r="C52" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D52" s="21">
+      <c r="D52" s="20">
         <v>1400</v>
       </c>
-      <c r="E52" s="15" t="s">
+      <c r="E52" s="14" t="s">
         <v>108</v>
       </c>
     </row>
@@ -2407,10 +2832,10 @@
       <c r="C53" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="D53" s="26">
+      <c r="D53" s="25">
         <v>1400</v>
       </c>
-      <c r="E53" s="15">
+      <c r="E53" s="14">
         <v>1404000586</v>
       </c>
     </row>
@@ -2421,10 +2846,10 @@
       <c r="C54" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="D54" s="25">
+      <c r="D54" s="24">
         <v>1400</v>
       </c>
-      <c r="E54" s="16">
+      <c r="E54" s="15">
         <v>1404000587</v>
       </c>
     </row>
@@ -2436,10 +2861,10 @@
       <c r="C55" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D55" s="21">
+      <c r="D55" s="20">
         <v>1900</v>
       </c>
-      <c r="E55" s="15" t="s">
+      <c r="E55" s="14" t="s">
         <v>109</v>
       </c>
     </row>
@@ -2451,10 +2876,10 @@
       <c r="C56" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D56" s="21">
+      <c r="D56" s="20">
         <v>1900</v>
       </c>
-      <c r="E56" s="15" t="s">
+      <c r="E56" s="14" t="s">
         <v>110</v>
       </c>
       <c r="F56">
@@ -2469,10 +2894,10 @@
       <c r="C57" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D57" s="21">
+      <c r="D57" s="20">
         <v>1900</v>
       </c>
-      <c r="E57" s="15" t="s">
+      <c r="E57" s="14" t="s">
         <v>111</v>
       </c>
     </row>
@@ -2483,10 +2908,10 @@
       <c r="C58" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="D58" s="25">
+      <c r="D58" s="24">
         <v>1900</v>
       </c>
-      <c r="E58" s="16">
+      <c r="E58" s="15">
         <v>1404000178</v>
       </c>
     </row>
@@ -2498,10 +2923,10 @@
       <c r="C59" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D59" s="21">
+      <c r="D59" s="20">
         <v>2400</v>
       </c>
-      <c r="E59" s="15" t="s">
+      <c r="E59" s="14" t="s">
         <v>112</v>
       </c>
     </row>
@@ -2513,10 +2938,10 @@
       <c r="C60" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D60" s="21">
+      <c r="D60" s="20">
         <v>2400</v>
       </c>
-      <c r="E60" s="15" t="s">
+      <c r="E60" s="14" t="s">
         <v>113</v>
       </c>
       <c r="F60">
@@ -2530,10 +2955,10 @@
       <c r="C61" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="D61" s="25">
+      <c r="D61" s="24">
         <v>2400</v>
       </c>
-      <c r="E61" s="16">
+      <c r="E61" s="15">
         <v>1404000234</v>
       </c>
     </row>
@@ -2545,10 +2970,10 @@
       <c r="C62" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D62" s="21">
+      <c r="D62" s="20">
         <v>3000</v>
       </c>
-      <c r="E62" s="15" t="s">
+      <c r="E62" s="14" t="s">
         <v>114</v>
       </c>
     </row>
@@ -2560,10 +2985,10 @@
       <c r="C63" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D63" s="21">
+      <c r="D63" s="20">
         <v>3000</v>
       </c>
-      <c r="E63" s="15" t="s">
+      <c r="E63" s="14" t="s">
         <v>115</v>
       </c>
       <c r="F63">
@@ -2577,10 +3002,10 @@
       <c r="C64" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="D64" s="27">
+      <c r="D64" s="26">
         <v>3000</v>
       </c>
-      <c r="E64" s="16">
+      <c r="E64" s="15">
         <v>1404000323</v>
       </c>
     </row>
@@ -2592,10 +3017,10 @@
       <c r="C65" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D65" s="21">
+      <c r="D65" s="20">
         <v>3600</v>
       </c>
-      <c r="E65" s="15" t="s">
+      <c r="E65" s="14" t="s">
         <v>116</v>
       </c>
       <c r="F65">
@@ -2609,10 +3034,10 @@
       <c r="C66" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="D66" s="27">
+      <c r="D66" s="26">
         <v>3600</v>
       </c>
-      <c r="E66" s="16">
+      <c r="E66" s="15">
         <v>1404000324</v>
       </c>
     </row>
@@ -2624,10 +3049,10 @@
       <c r="C67" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D67" s="21">
+      <c r="D67" s="20">
         <v>4300</v>
       </c>
-      <c r="E67" s="15" t="s">
+      <c r="E67" s="14" t="s">
         <v>118</v>
       </c>
       <c r="F67">
@@ -2641,10 +3066,10 @@
       <c r="C68" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="D68" s="27">
+      <c r="D68" s="26">
         <v>4300</v>
       </c>
-      <c r="E68" s="16">
+      <c r="E68" s="15">
         <v>1404000325</v>
       </c>
     </row>
@@ -2656,10 +3081,10 @@
       <c r="C69" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D69" s="21">
+      <c r="D69" s="20">
         <v>5000</v>
       </c>
-      <c r="E69" s="15" t="s">
+      <c r="E69" s="14" t="s">
         <v>119</v>
       </c>
       <c r="F69">
@@ -2673,10 +3098,10 @@
       <c r="C70" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="D70" s="27">
+      <c r="D70" s="26">
         <v>5000</v>
       </c>
-      <c r="E70" s="16">
+      <c r="E70" s="15">
         <v>1404000327</v>
       </c>
     </row>

</xml_diff>